<commit_message>
Update notebooks and inferences
</commit_message>
<xml_diff>
--- a/inferences/places-1701.xlsx
+++ b/inferences/places-1701.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>comment</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -474,8 +479,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Zhejiang， CHEKIANG (actuel ZHEJIANG)</t>
-        </is>
+          <t>Zhejiang 浙江， CHEKIANG (actuel ZHEJIANG)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="3">
@@ -501,8 +509,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hangzhou, </t>
-        </is>
+          <t xml:space="preserve">Hangzhou 杭州, </t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="4">
@@ -528,8 +539,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 海宁</t>
-        </is>
+          <t xml:space="preserve">海宁 </t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="5">
@@ -555,8 +569,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jiaxing, </t>
-        </is>
+          <t xml:space="preserve">Jiaxing 嘉兴, </t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="6">
@@ -582,8 +599,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jinhua, </t>
-        </is>
+          <t xml:space="preserve">Jinhua 金华, </t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="7">
@@ -609,8 +629,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lanxi, </t>
-        </is>
+          <t xml:space="preserve">Lanxi 兰溪, </t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="8">
@@ -636,8 +659,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ningbo, </t>
-        </is>
+          <t xml:space="preserve">Ningbo 宁波, </t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="9">
@@ -663,8 +689,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yinzhou, 鄞州 </t>
-        </is>
+          <t xml:space="preserve">Yinzhou 鄞州, </t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="10">
@@ -686,8 +715,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fujian, </t>
-        </is>
+          <t xml:space="preserve">Fujian 福建, </t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="11">
@@ -713,8 +745,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuzhou, </t>
-        </is>
+          <t xml:space="preserve">Fuzhou 福州, </t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="12">
@@ -740,8 +775,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lianjiang, </t>
-        </is>
+          <t xml:space="preserve">Lianjiang 连江, </t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="13">
@@ -767,8 +805,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zhangzhou, </t>
-        </is>
+          <t xml:space="preserve">Zhangzhou 漳州, </t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="14">
@@ -794,8 +835,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quanzhou, </t>
-        </is>
+          <t xml:space="preserve">Quanzhou 泉州, </t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="15">
@@ -821,8 +865,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xiamen, </t>
-        </is>
+          <t xml:space="preserve">Xiamen 厦门, </t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="16">
@@ -848,8 +895,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">(alors tcheou indépendant)Funing, </t>
-        </is>
+          <t>(alors tcheou indépendant)Funing, , hoje Xiapu 霞浦</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="17">
@@ -875,8 +925,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fu'an, </t>
-        </is>
+          <t xml:space="preserve">Fu'an 福安, </t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="18">
@@ -902,8 +955,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xinghua, </t>
-        </is>
+          <t>Xinghua 兴化, , 兴化县，the wikidata code of it dose not contain coordinate information, which can be substituted by Q68579，the present-day Putian 莆田</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="19">
@@ -929,8 +985,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kienning fou, Jianning, </t>
-        </is>
+          <t>Kienning fou, Jianning 建寧,  the wikidata code of it does not contain coordinate information, which can be substituted by Kien-yang today Jianyang Q639862 see 1644</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="20">
@@ -959,6 +1018,9 @@
           <t xml:space="preserve">浦城 </t>
         </is>
       </c>
+      <c r="F20" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -983,8 +1045,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shaowu, </t>
-        </is>
+          <t xml:space="preserve">Shaowu 邵武, </t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="22">
@@ -1010,8 +1075,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jianning Xian, </t>
-        </is>
+          <t xml:space="preserve">Jianning Xian 建宁, </t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="23">
@@ -1037,8 +1105,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tingzhou, </t>
-        </is>
+          <t xml:space="preserve">Tingzhou 汀州, </t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="24">
@@ -1067,6 +1138,9 @@
           <t xml:space="preserve">上杭 </t>
         </is>
       </c>
+      <c r="F24" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1091,8 +1165,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yanping, </t>
-        </is>
+          <t xml:space="preserve">Yanping 上杭, </t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="26">
@@ -1118,8 +1195,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jiangle 将乐</t>
-        </is>
+          <t xml:space="preserve">Jiangle 将乐, </t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="27">
@@ -1141,8 +1221,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Henan, </t>
-        </is>
+          <t xml:space="preserve">Henan 河南, </t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="28">
@@ -1168,8 +1251,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kaifeng, </t>
-        </is>
+          <t xml:space="preserve">Kaifeng 开封, </t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="29">
@@ -1195,8 +1281,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guide, </t>
-        </is>
+          <t>Guide, , hoje Shangqiu 商丘</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="30">
@@ -1218,8 +1307,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(actuel HUNAN + HUBEI)Huguang</t>
-        </is>
+          <t>湖广, (actuel HUNAN + HUBEI)Huguang</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="31">
@@ -1245,8 +1337,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wuchang, </t>
-        </is>
+          <t xml:space="preserve">Wuchang 武昌, </t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="32">
@@ -1272,8 +1367,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anlu, </t>
-        </is>
+          <t xml:space="preserve">Anlu 安陆, </t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="33">
@@ -1299,8 +1397,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 长沙</t>
-        </is>
+          <t xml:space="preserve">长沙 </t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="34">
@@ -1326,8 +1427,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Xiangtan,湘潭</t>
-        </is>
+          <t xml:space="preserve">Xiangtan 湘潭, </t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="35">
@@ -1353,8 +1457,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Chenzhou，郴州 Chen(g)chow</t>
-        </is>
+          <t>Chenzhou 郴州, Chen(g)chow</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="36">
@@ -1380,8 +1487,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>, Hengyang</t>
-        </is>
+          <t xml:space="preserve">Hengyang 衡阳, </t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="37">
@@ -1407,8 +1517,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jingzhou, </t>
-        </is>
+          <t xml:space="preserve">Jingzhou 荆州, </t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="38">
@@ -1437,6 +1550,9 @@
           <t>No Wikidata</t>
         </is>
       </c>
+      <c r="F38" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1461,8 +1577,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yongzhou, </t>
-        </is>
+          <t xml:space="preserve">Yongzhou 永州, </t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="40">
@@ -1484,8 +1603,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">KIANGNAN ou NANKIN (actuel ANHUI + JIANGSU),Jiangnan, </t>
-        </is>
+          <t xml:space="preserve">KIANGNAN ou NANKIN (actuel ANHUI + JIANGSU),Jiangnan 江南, </t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="41">
@@ -1511,8 +1633,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nanjing, </t>
-        </is>
+          <t xml:space="preserve">Nanjing 南京, </t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="42">
@@ -1533,13 +1658,16 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>No wikidata</t>
+          <t>Q360374</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>wikidata:Q360374,Anqing, 安庆</t>
-        </is>
+          <t xml:space="preserve">Anqing 安庆, </t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="43">
@@ -1565,8 +1693,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Changzhou, </t>
-        </is>
+          <t xml:space="preserve">Changzhou 常州, </t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="44">
@@ -1592,8 +1723,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wuxi, 无锡, </t>
-        </is>
+          <t xml:space="preserve">Wuxi 无锡, </t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="45">
@@ -1619,8 +1753,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Chizhou, 池州Chinchow (= Kweichih)</t>
-        </is>
+          <t>Chizhou 池州, Chinchow (= Kweichih)</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="46">
@@ -1646,8 +1783,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zhenjiang, </t>
-        </is>
+          <t xml:space="preserve">Zhenjiang 镇江, </t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="47">
@@ -1673,8 +1813,11 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Danyang, </t>
-        </is>
+          <t xml:space="preserve">Danyang 丹阳, </t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="48">
@@ -1700,8 +1843,11 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 凤阳</t>
-        </is>
+          <t xml:space="preserve">凤阳, </t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="49">
@@ -1727,8 +1873,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>.Wuhe, 五河</t>
-        </is>
+          <t xml:space="preserve">Wuhe 五河, </t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="50">
@@ -1754,8 +1903,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huai'an, </t>
-        </is>
+          <t xml:space="preserve">Huai'an 淮安, </t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="51">
@@ -1776,13 +1928,16 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Q57719</t>
+          <t>Q42622</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Xuzhou, 徐州</t>
-        </is>
+          <t xml:space="preserve">Suzhou 苏州, </t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="52">
@@ -1808,8 +1963,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Changshu (Cham xo), Changshu, </t>
-        </is>
+          <t xml:space="preserve">Changshu (Cham xo), Changshu 常熟, </t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="53">
@@ -1835,8 +1993,11 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>,Kunshan, 昆山</t>
-        </is>
+          <t xml:space="preserve">昆山, </t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="54">
@@ -1857,13 +2018,16 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Q42622</t>
+          <t>Q57719</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suzhou, </t>
-        </is>
+          <t xml:space="preserve">Xuzhou 徐州, </t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="55">
@@ -1889,8 +2053,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Songjiang, </t>
-        </is>
+          <t xml:space="preserve">Songjiang 松江, </t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="56">
@@ -1916,8 +2083,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shanghai, </t>
-        </is>
+          <t xml:space="preserve">Shanghai 上海, </t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="57">
@@ -1946,6 +2116,9 @@
           <t xml:space="preserve">Qingpu, </t>
         </is>
       </c>
+      <c r="F57" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1970,8 +2143,11 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Taicang, 太仓</t>
-        </is>
+          <t xml:space="preserve">Taicang 太仓, </t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="59">
@@ -1997,8 +2173,11 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jiading, </t>
-        </is>
+          <t xml:space="preserve">Jiading 嘉定, </t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="60">
@@ -2024,8 +2203,11 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chongming, </t>
-        </is>
+          <t xml:space="preserve">Chongming 崇明, </t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="61">
@@ -2051,8 +2233,11 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yangzhou, </t>
-        </is>
+          <t xml:space="preserve">Yangzhou 扬州, </t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="62">
@@ -2074,8 +2259,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jiangxi, </t>
-        </is>
+          <t xml:space="preserve">Jiangxi 江西, </t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="63">
@@ -2101,8 +2289,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nanchang, </t>
-        </is>
+          <t xml:space="preserve">Nanchang 南昌, </t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="64">
@@ -2128,8 +2319,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>, Fuzhou, 抚州</t>
-        </is>
+          <t xml:space="preserve">Fuzhou 抚州, </t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="65">
@@ -2155,8 +2349,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Raozhou, 饶州,present day Poyang County</t>
-        </is>
+          <t>Raozhou 饶州, , present day Poyang County</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="66">
@@ -2185,6 +2382,9 @@
           <t xml:space="preserve">Ganzhou (赣州) in Jiangxi </t>
         </is>
       </c>
+      <c r="F66" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2209,8 +2409,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>,Ningdu, 宁都</t>
-        </is>
+          <t xml:space="preserve">Ningdu 宁都, </t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="68">
@@ -2236,8 +2439,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>, Xinfeng,信丰</t>
-        </is>
+          <t xml:space="preserve">Xinfeng 信丰, </t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="69">
@@ -2263,8 +2469,11 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>,Ji'an,吉安</t>
-        </is>
+          <t xml:space="preserve">Ji'an 吉安, </t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="70">
@@ -2290,8 +2499,11 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>, Dingnan, 定南</t>
-        </is>
+          <t xml:space="preserve">Dingnan 定南, </t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="71">
@@ -2317,8 +2529,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jianchang, </t>
-        </is>
+          <t xml:space="preserve">Jianchang 建昌, </t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="72">
@@ -2344,8 +2559,11 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nanfeng, </t>
-        </is>
+          <t xml:space="preserve">Nanfeng 南丰, </t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="73">
@@ -2371,8 +2589,11 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>,Jiujiang, 九江</t>
-        </is>
+          <t xml:space="preserve">Jiujiang 九江, </t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="74">
@@ -2398,8 +2619,11 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Guangxin, 广信</t>
-        </is>
+          <t xml:space="preserve">Guangxin 广信, </t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="75">
@@ -2425,8 +2649,11 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>,Yushan, 玉山</t>
-        </is>
+          <t xml:space="preserve">玉山, </t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="76">
@@ -2452,8 +2679,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nan'an, </t>
-        </is>
+          <t xml:space="preserve">Nan'an 南安, </t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="77">
@@ -2482,6 +2712,9 @@
           <t>No wikidata</t>
         </is>
       </c>
+      <c r="F77" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2502,8 +2735,11 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guangxi, </t>
-        </is>
+          <t xml:space="preserve">Guangxi 广西, </t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="79">
@@ -2529,8 +2765,11 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guilin, </t>
-        </is>
+          <t xml:space="preserve">Guilin 桂林, </t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="80">
@@ -2556,8 +2795,11 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wuzhou, </t>
-        </is>
+          <t xml:space="preserve">Wuzhou 梧州, </t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="81">
@@ -2579,8 +2821,11 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guangdong, </t>
-        </is>
+          <t xml:space="preserve">Guangdong 广东, </t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="82">
@@ -2606,8 +2851,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>,Guangzhou, 广州Canton</t>
-        </is>
+          <t>Guangzhou 广州, Canton</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="83">
@@ -2633,8 +2881,11 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>,Foshan, 佛山</t>
-        </is>
+          <t xml:space="preserve">Foshan 佛山, </t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="84">
@@ -2655,13 +2906,16 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>No wikidata</t>
+          <t>Q1023903</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>wikidata:Q1023903,Xinhui, 新会</t>
-        </is>
+          <t xml:space="preserve">Xinhui 新会, </t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="85">
@@ -2687,8 +2941,11 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dongguan, </t>
-        </is>
+          <t xml:space="preserve">Dongguan 东莞, </t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="86">
@@ -2714,8 +2971,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiungchow (île de Hainan), Qiongzhou, </t>
-        </is>
+          <t>琼州, Kiungchow (île de Hainan), Qiongzhou</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="87">
@@ -2741,8 +3001,11 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>, Lianzhou, 廉州 present day Hepu County</t>
-        </is>
+          <t>Lianzhou 廉州, , present day Hepu County</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="88">
@@ -2768,8 +3031,11 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leizhou, </t>
-        </is>
+          <t xml:space="preserve">Leizhou 雷州, </t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="89">
@@ -2795,8 +3061,11 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nanxiong, </t>
-        </is>
+          <t xml:space="preserve">Nanxiong 南雄, </t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="90">
@@ -2822,8 +3091,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Shixing, 始兴</t>
-        </is>
+          <t xml:space="preserve">Shixing 始兴, </t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="91">
@@ -2849,8 +3121,11 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>,Shuntak (Xunte Shunde, 顺德Shuntak (Xunte)</t>
-        </is>
+          <t xml:space="preserve">Xunte Shunde 顺德, </t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="92">
@@ -2879,6 +3154,9 @@
           <t>No wikidataShiuhow (Xao cheu)</t>
         </is>
       </c>
+      <c r="F92" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2903,8 +3181,11 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>,Lecong, 乐从</t>
-        </is>
+          <t xml:space="preserve">Lecong 乐从, </t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="94">
@@ -2933,6 +3214,9 @@
           <t>No wikidataYanfa -- Gin hoa</t>
         </is>
       </c>
+      <c r="F94" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2957,8 +3241,11 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chao Kim, Zhaoqing, </t>
-        </is>
+          <t xml:space="preserve">Chao Kim, Zhaoqing 肇庆, </t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="96">
@@ -2984,8 +3271,11 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>,Huizhou,惠州Waichow, Hwaichow (Hoei cheu), Guizhou,</t>
-        </is>
+          <t>Huizhou,惠州 Waichow, Hwaichow (Hoei cheu), Guizhou,</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="97">
@@ -3010,6 +3300,9 @@
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
+      <c r="F97" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3037,6 +3330,9 @@
           <t xml:space="preserve">Ilha Verde, </t>
         </is>
       </c>
+      <c r="F98" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3064,6 +3360,9 @@
           <t xml:space="preserve">Lapa (Wan-tchai),Wanzai, </t>
         </is>
       </c>
+      <c r="F99" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3084,8 +3383,11 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">KWEICHOW (actuel GUIZHOU): néant Guizhou, </t>
-        </is>
+          <t xml:space="preserve">KWEICHOW (actuel GUIZHOU): néant Guizhou 贵州, </t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="101">
@@ -3107,8 +3409,11 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>PEKING (actuel HEBEI)</t>
-        </is>
+          <t>PEKING (actuel HEBEI) 北京</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="102">
@@ -3134,8 +3439,11 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pékin collège St Joseph (1605) ou Si-t'ang (sera appelé Nan-t'ang en 1723, à cause du Si-t'ang fondé pour la Propagande, R), Beijing, </t>
-        </is>
+          <t>Beijing 北京, Pékin collège St Joseph (1605) ou Si-t'ang (sera appelé Nan-t'ang en 1723, à cause du Si-t'ang fondé pour la Propagande, R)</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="103">
@@ -3161,8 +3469,11 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 西堂Si-t'ang fondé pour la Propagande, R [em 1703])</t>
-        </is>
+          <t>Xitang 西堂  西堂Si-t'ang fondé pour la Propagande, R [em 1703])</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="104">
@@ -3188,8 +3499,11 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 东堂Tong-t'ang ou R Saint-Joseph (1655)</t>
-        </is>
+          <t>Dongtang 东堂  东堂Tong-t'ang ou R Saint-Joseph (1655)</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="105">
@@ -3215,8 +3529,11 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 北堂</t>
-        </is>
+          <t xml:space="preserve">Beitang, 北堂 </t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="106">
@@ -3242,8 +3559,11 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Liangxiang, 良乡</t>
-        </is>
+          <t xml:space="preserve">Liangxiang 良乡, </t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="107">
@@ -3269,8 +3589,11 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tongzhou, </t>
-        </is>
+          <t xml:space="preserve">Tongzhou 通州, </t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="108">
@@ -3296,8 +3619,11 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zhengding, </t>
-        </is>
+          <t xml:space="preserve">Zhengding 正定, </t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="109">
@@ -3323,8 +3649,11 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baoding, </t>
-        </is>
+          <t xml:space="preserve">Baoding 保定, </t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="110">
@@ -3346,8 +3675,11 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shanxi, </t>
-        </is>
+          <t xml:space="preserve">Shanxi 山西, </t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="111">
@@ -3373,8 +3705,11 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taiyuan, </t>
-        </is>
+          <t xml:space="preserve">Taiyuan 太原, </t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="112">
@@ -3400,8 +3735,11 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>,Fenzhou, 汾州</t>
-        </is>
+          <t xml:space="preserve">Fenzhou 汾州, </t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="113">
@@ -3427,8 +3765,11 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>, 平遥Pingyao du Fenchow</t>
-        </is>
+          <t xml:space="preserve">Pingyao du Fenchow 平遥, </t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="114">
@@ -3454,8 +3795,11 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jiexiu, 介休Kiehsiu du Fenchow</t>
-        </is>
+          <t>Jiexiu 介休, Kiehsiu du Fenchow</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="115">
@@ -3484,6 +3828,9 @@
           <t>Pingyang Fu, , Q73156</t>
         </is>
       </c>
+      <c r="F115" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3511,6 +3858,9 @@
           <t xml:space="preserve">Jiangzhou, </t>
         </is>
       </c>
+      <c r="F116" t="n">
+        <v>1701</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3535,8 +3885,11 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzhou, </t>
-        </is>
+          <t xml:space="preserve">Puzhou 绛州, </t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="118">
@@ -3557,13 +3910,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Q1197616</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 洪洞</t>
-        </is>
+          <t>No wikidata</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="119">
@@ -3579,18 +3931,21 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Kiehsiu</t>
+          <t>Siangling</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Q1362530</t>
+          <t>Q22099543</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Jiexiu, 介休</t>
-        </is>
+          <t xml:space="preserve">Xiangling 襄陵县，the wikidata code of it does not contain coordination information, which can be substituted by Q1197358，present day Xiangfen County 襄汾县, </t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="120">
@@ -3606,18 +3961,21 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Siangling</t>
+          <t>Taiping</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Q22099543</t>
+          <t>Q18111423</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Xiangling 襄陵县，the wikidata code of it dose not contain coordination information, which can be substituted by Q1197358，present day Xiangfen County 襄汾县</t>
-        </is>
+          <t>Taiping 太平县，the wikidata code of it does not contain coordinate information, which can be substituted by Q11137509，the present-day 汾城镇 , , Q1113750</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="121">
@@ -3633,18 +3991,21 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Taiping</t>
+          <t>Wanchuan</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Q18111423</t>
+          <t>Q8475332</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Taiping, ,太平县，the wikidata code of it dose not contain coordinate information, which can be substituted by Q11137509，the present-day 汾城镇</t>
-        </is>
+          <t xml:space="preserve">Wanquan 万泉县，the wikidata code of it does not contain coordinate information, which can be substituted by Q1196908，the present-day万荣县, </t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="122">
@@ -3655,23 +4016,26 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Pingyang</t>
+          <t>Sinchow</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Wanchuan</t>
+          <t>Sinchow</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Q8475332</t>
+          <t>Q73119</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 万泉县，the wikidata code of it dose not contain coordinate information, which can be substituted by Q1196908，the present-day万荣县</t>
-        </is>
+          <t xml:space="preserve">Xinzhou 忻州, </t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="123">
@@ -3687,45 +4051,47 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Sinchow</t>
+          <t>Tsinglo</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Q73119</t>
+          <t>Q174034</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>,Xinzhou, 忻州</t>
-        </is>
+          <t xml:space="preserve">Jingle 静乐, </t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Shansi</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Sinchow</t>
-        </is>
-      </c>
+          <t>Shantung</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Tsinglo</t>
+          <t>Shantung</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Q174034</t>
+          <t>Q43407</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>,Jingle, 静乐</t>
-        </is>
+          <t xml:space="preserve">actuel Shandong, Shandong 山东, </t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="125">
@@ -3734,21 +4100,28 @@
           <t>Shantung</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Tsinan</t>
+        </is>
+      </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Shantung</t>
+          <t>Tsinan</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Q43407</t>
+          <t>Q170247</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t xml:space="preserve">actuel Shandong, Shandong, </t>
-        </is>
+          <t xml:space="preserve">Jinan 济南, </t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="126">
@@ -3764,18 +4137,21 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Tsinan</t>
+          <t>Taian</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Q170247</t>
+          <t>Q217681</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jinan, </t>
-        </is>
+          <t xml:space="preserve">Tai'an 泰安, </t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="127">
@@ -3791,18 +4167,21 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Taian</t>
+          <t>Tehchow</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Q217681</t>
+          <t>Q162880</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tai'an, </t>
-        </is>
+          <t xml:space="preserve">Dezhou 德州, </t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="128">
@@ -3813,23 +4192,26 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Tsinan</t>
+          <t>Tsingchow</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Tehchow</t>
+          <t>Tsingchow</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Q162880</t>
+          <t>Q1360781</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>,Dezhou,德州</t>
-        </is>
+          <t xml:space="preserve">(-- Idu, Yitu)Qingzhou 青州, , Yidu, </t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="129">
@@ -3840,23 +4222,26 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Tsingchow</t>
+          <t>Linchu</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Tsingchow</t>
+          <t>Linchu</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Q1360781</t>
+          <t>Q1198208</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t xml:space="preserve">(-- Idu, Yitu)Qingzhou, , Yidu, </t>
-        </is>
+          <t xml:space="preserve">Linkiu 临朐, </t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="130">
@@ -3867,23 +4252,26 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Linchu</t>
+          <t>Tungchang</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Linchu</t>
+          <t>Tungchang</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Q1198208</t>
+          <t>Q10870440</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>,Linkiu, 临朐</t>
-        </is>
+          <t xml:space="preserve">Dungchang 东昌, </t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="131">
@@ -3899,18 +4287,21 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Tungchang</t>
+          <t>Lintsing</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Q10870440</t>
+          <t>Q1207099</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dungchang, </t>
-        </is>
+          <t xml:space="preserve">Linqing 临清, </t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="132">
@@ -3921,23 +4312,26 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tungchang</t>
+          <t>Yenchow</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Lintsing</t>
+          <t>Yenchow</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>No wikidata</t>
+          <t>Q10891140</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>wikidata:Q1207099.Linqing, 临清</t>
-        </is>
+          <t xml:space="preserve">Yanzhou 兖州, </t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="133">
@@ -3953,18 +4347,21 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Yenchow</t>
+          <t>Ichow</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Q10891140</t>
+          <t>Q11552388</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Yanzhou, 兖州</t>
-        </is>
+          <t>(hoje Linyi, Shandong) 沂州, Ichow (-- Lini), alors tcheou</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="134">
@@ -3980,45 +4377,47 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Ichow</t>
+          <t>Tsining</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Q11552388</t>
+          <t>Q372791</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Ichow ( -- Lini)</t>
-        </is>
+          <t xml:space="preserve">Jining 济宁, </t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Shantung</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>Yenchow</t>
-        </is>
-      </c>
+          <t>Shensi</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Tsining</t>
+          <t>Shensi</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Q372791</t>
+          <t>Q46913</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>,Jining, 济宁</t>
-        </is>
+          <t>Hoje Shaanxi para distinguir de deh-r1701-shansi (actuel SHANXI)Shanxi</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="136">
@@ -4027,21 +4426,28 @@
           <t>Shensi</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Sian</t>
+        </is>
+      </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Shensi</t>
+          <t>Sian</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Q46913</t>
+          <t>Q5826</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>(actuel SHANXI)Shanxi,  Shaanxi 陕西</t>
-        </is>
+          <t xml:space="preserve">Xi'an 西安, </t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="137">
@@ -4057,18 +4463,21 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Sian</t>
+          <t>Sanyuan</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Q5826</t>
+          <t>Q1201362</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xi'an, </t>
-        </is>
+          <t xml:space="preserve">Sanyuan 三原, </t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="138">
@@ -4079,23 +4488,26 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sian</t>
+          <t>Hanchung</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Sanyuan</t>
+          <t>Hanchung</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Q1201362</t>
+          <t>Q515573</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sanyuan, </t>
-        </is>
+          <t xml:space="preserve">Hanzhong 汉中, </t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="139">
@@ -4106,23 +4518,26 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Hanchung</t>
+          <t>Chengku</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Hanchung</t>
+          <t>Chengku</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Q515573</t>
+          <t>Q1069968</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hanzhong, </t>
-        </is>
+          <t xml:space="preserve">Chenggu 城固, </t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="140">
@@ -4138,45 +4553,47 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Chengku</t>
+          <t>Siao-tchai</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Q1069968</t>
+          <t>No wikidata</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chenggu, </t>
-        </is>
+          <t>No wikidataSiao-tchai du Chengku</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Shensi</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Chengku</t>
-        </is>
-      </c>
+          <t>Szechwan</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Siao-tchai</t>
+          <t>Szechwan</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>No wikidata</t>
+          <t>Q19770</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>No wikidataSiao-tchai du Chengku</t>
-        </is>
+          <t xml:space="preserve">actuel SICHUAN)Sichuan 四川, </t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="142">
@@ -4185,21 +4602,28 @@
           <t>Szechwan</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Chengtu</t>
+        </is>
+      </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Szechwan</t>
+          <t>Chengtu</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Q19770</t>
+          <t>Q30002</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t xml:space="preserve">actuel SICHUAN)Sichuan, </t>
-        </is>
+          <t xml:space="preserve">Chengdu 成都, </t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="143">
@@ -4210,50 +4634,52 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Chengtu</t>
+          <t>Chungking</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Chengtu</t>
+          <t>Chungking</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Q30002</t>
+          <t>Q11725</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chengdu, </t>
-        </is>
+          <t xml:space="preserve">Chongqing 重庆, </t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Szechwan</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Chungking</t>
-        </is>
-      </c>
+          <t>Yunnan</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Chungking</t>
+          <t>Yunnan</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Q11725</t>
+          <t>Q43194</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chongqing, </t>
-        </is>
+          <t xml:space="preserve">Yunnan 云南, </t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>1701</v>
       </c>
     </row>
     <row r="145">
@@ -4262,45 +4688,29 @@
           <t>Yunnan</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Yunnanfu</t>
+        </is>
+      </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Yunnan</t>
+          <t>Yunnanfu</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Q43194</t>
+          <t>Q182852</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yunnan, </t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Yunnan</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Yunnanfu</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>Yunnanfu</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>No wikidata</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr"/>
+          <t xml:space="preserve">Yunanfu,present day Kunming 昆明, </t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>1701</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>